<commit_message>
Adiciona fabricante (opcional) ao cadastro de item
Novo campo de texto livre, nunca obrigatorio, no cadastro do item
(tela Estoque, script de importacao por planilha e API). Atualiza
tambem o modelo de planilha (docs/modelo_importacao_itens.xlsx) com a
coluna nova, mesmo padrao visual (verde = opcional) das demais.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/modelo_importacao_itens.xlsx
+++ b/docs/modelo_importacao_itens.xlsx
@@ -101,7 +101,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -114,6 +114,8 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -204,6 +206,11 @@
     <comment ref="F1" authorId="0" shapeId="0">
       <text>
         <t>Verde = coluna opcional (só pra já registrar estoque inicial). Ver aba 'Instruções'.</t>
+      </text>
+    </comment>
+    <comment ref="K1" authorId="0" shapeId="0">
+      <text>
+        <t>Opcional — vira o campo "Fabricante" do cadastro do item (não do lote). Ver aba 'Instruções'.</t>
       </text>
     </comment>
   </commentList>
@@ -499,7 +506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J26"/>
+  <dimension ref="A1:K26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -512,6 +519,7 @@
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -565,6 +573,11 @@
           <t>numero_nota_fiscal</t>
         </is>
       </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>fabricante</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -609,6 +622,11 @@
       <c r="J2" s="3" t="inlineStr">
         <is>
           <t>NF-00123</t>
+        </is>
+      </c>
+      <c r="K2" s="3" t="inlineStr">
+        <is>
+          <t>Descarpack</t>
         </is>
       </c>
     </row>
@@ -647,6 +665,11 @@
       <c r="J3" s="3" t="inlineStr">
         <is>
           <t>NF-00123</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>3M</t>
         </is>
       </c>
     </row>
@@ -679,6 +702,11 @@
       <c r="H4" s="3" t="n"/>
       <c r="I4" s="3" t="n"/>
       <c r="J4" s="3" t="n"/>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>Rioquimica</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -709,6 +737,11 @@
       <c r="H5" s="3" t="n"/>
       <c r="I5" s="3" t="n"/>
       <c r="J5" s="3" t="n"/>
+      <c r="K5" s="3" t="inlineStr">
+        <is>
+          <t>Faber-Castell</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n"/>
@@ -721,6 +754,7 @@
       <c r="H6" s="4" t="n"/>
       <c r="I6" s="4" t="n"/>
       <c r="J6" s="4" t="n"/>
+      <c r="K6" s="8" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n"/>
@@ -733,6 +767,7 @@
       <c r="H7" s="4" t="n"/>
       <c r="I7" s="4" t="n"/>
       <c r="J7" s="4" t="n"/>
+      <c r="K7" s="8" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n"/>
@@ -745,6 +780,7 @@
       <c r="H8" s="4" t="n"/>
       <c r="I8" s="4" t="n"/>
       <c r="J8" s="4" t="n"/>
+      <c r="K8" s="8" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n"/>
@@ -757,6 +793,7 @@
       <c r="H9" s="4" t="n"/>
       <c r="I9" s="4" t="n"/>
       <c r="J9" s="4" t="n"/>
+      <c r="K9" s="8" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n"/>
@@ -769,6 +806,7 @@
       <c r="H10" s="4" t="n"/>
       <c r="I10" s="4" t="n"/>
       <c r="J10" s="4" t="n"/>
+      <c r="K10" s="8" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n"/>
@@ -781,6 +819,7 @@
       <c r="H11" s="4" t="n"/>
       <c r="I11" s="4" t="n"/>
       <c r="J11" s="4" t="n"/>
+      <c r="K11" s="8" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n"/>
@@ -793,6 +832,7 @@
       <c r="H12" s="4" t="n"/>
       <c r="I12" s="4" t="n"/>
       <c r="J12" s="4" t="n"/>
+      <c r="K12" s="8" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n"/>
@@ -805,6 +845,7 @@
       <c r="H13" s="4" t="n"/>
       <c r="I13" s="4" t="n"/>
       <c r="J13" s="4" t="n"/>
+      <c r="K13" s="8" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n"/>
@@ -817,6 +858,7 @@
       <c r="H14" s="4" t="n"/>
       <c r="I14" s="4" t="n"/>
       <c r="J14" s="4" t="n"/>
+      <c r="K14" s="8" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n"/>
@@ -829,6 +871,7 @@
       <c r="H15" s="4" t="n"/>
       <c r="I15" s="4" t="n"/>
       <c r="J15" s="4" t="n"/>
+      <c r="K15" s="8" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n"/>
@@ -841,6 +884,7 @@
       <c r="H16" s="4" t="n"/>
       <c r="I16" s="4" t="n"/>
       <c r="J16" s="4" t="n"/>
+      <c r="K16" s="8" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n"/>
@@ -853,6 +897,7 @@
       <c r="H17" s="4" t="n"/>
       <c r="I17" s="4" t="n"/>
       <c r="J17" s="4" t="n"/>
+      <c r="K17" s="8" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n"/>
@@ -865,6 +910,7 @@
       <c r="H18" s="4" t="n"/>
       <c r="I18" s="4" t="n"/>
       <c r="J18" s="4" t="n"/>
+      <c r="K18" s="8" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n"/>
@@ -877,6 +923,7 @@
       <c r="H19" s="4" t="n"/>
       <c r="I19" s="4" t="n"/>
       <c r="J19" s="4" t="n"/>
+      <c r="K19" s="8" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n"/>
@@ -889,6 +936,7 @@
       <c r="H20" s="4" t="n"/>
       <c r="I20" s="4" t="n"/>
       <c r="J20" s="4" t="n"/>
+      <c r="K20" s="8" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n"/>
@@ -901,6 +949,7 @@
       <c r="H21" s="4" t="n"/>
       <c r="I21" s="4" t="n"/>
       <c r="J21" s="4" t="n"/>
+      <c r="K21" s="8" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n"/>
@@ -913,6 +962,7 @@
       <c r="H22" s="4" t="n"/>
       <c r="I22" s="4" t="n"/>
       <c r="J22" s="4" t="n"/>
+      <c r="K22" s="8" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n"/>
@@ -925,6 +975,7 @@
       <c r="H23" s="4" t="n"/>
       <c r="I23" s="4" t="n"/>
       <c r="J23" s="4" t="n"/>
+      <c r="K23" s="8" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="4" t="n"/>
@@ -937,6 +988,7 @@
       <c r="H24" s="4" t="n"/>
       <c r="I24" s="4" t="n"/>
       <c r="J24" s="4" t="n"/>
+      <c r="K24" s="8" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n"/>
@@ -949,6 +1001,7 @@
       <c r="H25" s="4" t="n"/>
       <c r="I25" s="4" t="n"/>
       <c r="J25" s="4" t="n"/>
+      <c r="K25" s="8" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="4" t="n"/>
@@ -961,6 +1014,7 @@
       <c r="H26" s="4" t="n"/>
       <c r="I26" s="4" t="n"/>
       <c r="J26" s="4" t="n"/>
+      <c r="K26" s="8" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -974,7 +1028,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A39"/>
+  <dimension ref="A1:A41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -1114,76 +1168,80 @@
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>"dar entrada" depois pela tela Entrada por Compra):</t>
+          <t>"dar entrada" depois pela tela Entrada por Compra. fabricante é a exceção: não tem</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • quantidade — número inteiro; SE preenchida, cria automaticamente uma entrada de estoque</t>
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>relação com estoque, é só um dado a mais do cadastro do item, sempre opcional):</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • numero_lote — texto, opcional mesmo com quantidade preenchida</t>
+          <t xml:space="preserve">  • quantidade — número inteiro; SE preenchida, cria automaticamente uma entrada de estoque</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • data_validade — formato AAAA-MM-DD (ex.: 2027-01-15); deixe em branco se o item não vence</t>
+          <t xml:space="preserve">  • numero_lote — texto, opcional mesmo com quantidade preenchida</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • valor_unitario — número com ponto decimal (ex.: 3.50, não 3,50)</t>
+          <t xml:space="preserve">  • data_validade — formato AAAA-MM-DD (ex.: 2027-01-15); deixe em branco se o item não vence</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
+          <t xml:space="preserve">  • valor_unitario — número com ponto decimal (ex.: 3.50, não 3,50)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
           <t xml:space="preserve">  • numero_nota_fiscal — texto</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="6" t="inlineStr"/>
-    </row>
     <row r="29">
-      <c r="A29" s="6" t="inlineStr">
-        <is>
-          <t>As linhas 2 a 5 (fundo amarelo) são EXEMPLOS de preenchimento — apague-as antes de importar</t>
+      <c r="A29" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • fabricante — texto (ex.: 3M, Descarpack); vira o cadastro do ITEM, não do lote</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="6" t="inlineStr">
-        <is>
-          <t>de verdade, ou deixe (o script pula automaticamente porque esses códigos já existem no</t>
-        </is>
-      </c>
+      <c r="A30" s="6" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
+          <t>As linhas 2 a 5 (fundo amarelo) são EXEMPLOS de preenchimento — apague-as antes de importar</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>de verdade, ou deixe (o script pula automaticamente porque esses códigos já existem no</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
           <t>catálogo de exemplo do ambiente de teste).</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="6" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="7" t="inlineStr">
-        <is>
-          <t>COMO RODAR (a partir da pasta backend/, com o ambiente já configurado):</t>
         </is>
       </c>
     </row>
@@ -1191,31 +1249,41 @@
       <c r="A34" s="6" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="6" t="inlineStr">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>COMO RODAR (a partir da pasta backend/, com o ambiente já configurado):</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  python scripts/importar_itens_planilha.py caminho/modelo_importacao_itens.xlsx \</t>
         </is>
       </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      --api-url http://localhost:8000 --login coordenador --senha "sua-senha"</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="6" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
+          <t xml:space="preserve">      --api-url http://localhost:8000 --login coordenador --senha "sua-senha"</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="inlineStr">
+        <is>
           <t>Ver docs/05_INSTALACAO_SERVIDOR_LOCAL.md para o passo completo dentro do processo de</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="6" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="6" t="inlineStr">
         <is>
           <t>instalação.</t>
         </is>

</xml_diff>

<commit_message>
Estoque minimo deixa de ser obrigatorio; importacao passa a incluir setores
- estoque_minimo agora e opcional no cadastro/edicao de item (frontend
  e script de importacao) -- backend ja tratava como default 0.
- importar_itens_planilha.py ganha --setores: importa uma planilha de
  setores separada da de itens (so uma coluna, nome), idempotente do
  mesmo jeito, podendo rodar junto com a importacao de itens ou sozinho.
- modelo_importacao_itens.xlsx e docs atualizados de acordo.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/modelo_importacao_itens.xlsx
+++ b/docs/modelo_importacao_itens.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Itens" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Instruções" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Itens" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instruções" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -201,6 +201,11 @@
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
         <t>Azul = coluna obrigatória. Ver aba 'Instruções' para o detalhe completo.</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>Opcional — 0 se deixar em branco ou preencher errado. Ver aba 'Instruções'.</t>
       </text>
     </comment>
     <comment ref="F1" authorId="0" shapeId="0">
@@ -543,7 +548,7 @@
           <t>categoria</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>estoque_minimo</t>
         </is>
@@ -1028,7 +1033,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A41"/>
+  <dimension ref="A1:A42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -1104,186 +1109,193 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • estoque_minimo — número inteiro (use 0 se ainda não souber)</t>
-        </is>
-      </c>
+      <c r="A12" s="6" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="inlineStr"/>
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>CATEGORIAS ACEITAS (qualquer uma das grafias abaixo funciona, sem diferenciar maiúscula/acento):</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="inlineStr">
-        <is>
-          <t>CATEGORIAS ACEITAS (qualquer uma das grafias abaixo funciona, sem diferenciar maiúscula/acento):</t>
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Material Médico  →  também aceita: material_medico, Mat. Med.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Material Médico  →  também aceita: material_medico, Mat. Med.</t>
+          <t xml:space="preserve">  • EPI  →  também aceita: EPI/SIAST</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • EPI  →  também aceita: EPI/SIAST</t>
+          <t xml:space="preserve">  • Higienização  →  também aceita: Higienizacao</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Higienização  →  também aceita: Higienizacao</t>
+          <t xml:space="preserve">  • Material de Expediente  →  também aceita: Expediente</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Material de Expediente  →  também aceita: Expediente</t>
-        </is>
-      </c>
+      <c r="A18" s="6" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="inlineStr"/>
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>COLUNAS OPCIONAIS (fundo verde no cabeçalho — preencha só se já tiver estoque desse item</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>COLUNAS OPCIONAIS (fundo verde no cabeçalho — preencha só se já tiver estoque desse item</t>
+          <t>pra registrar junto com o cadastro; deixando em branco, o item nasce com saldo 0 e dá pra</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="6" t="inlineStr">
-        <is>
-          <t>pra registrar junto com o cadastro; deixando em branco, o item nasce com saldo 0 e dá pra</t>
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>"dar entrada" depois pela tela Entrada por Compra. estoque_minimo e fabricante são</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="7" t="inlineStr">
-        <is>
-          <t>"dar entrada" depois pela tela Entrada por Compra. fabricante é a exceção: não tem</t>
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>as exceções: não têm relação com estoque, são só dados a mais do cadastro do item,</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="9" t="inlineStr">
         <is>
-          <t>relação com estoque, é só um dado a mais do cadastro do item, sempre opcional):</t>
+          <t>sempre opcionais):</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • quantidade — número inteiro; SE preenchida, cria automaticamente uma entrada de estoque</t>
+      <c r="A24" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • estoque_minimo — número inteiro; 0 se deixar em branco ou preencher algo que não é número</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • numero_lote — texto, opcional mesmo com quantidade preenchida</t>
+          <t xml:space="preserve">  • quantidade — número inteiro; SE preenchida, cria automaticamente uma entrada de estoque</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • data_validade — formato AAAA-MM-DD (ex.: 2027-01-15); deixe em branco se o item não vence</t>
+          <t xml:space="preserve">  • numero_lote — texto, opcional mesmo com quantidade preenchida</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • valor_unitario — número com ponto decimal (ex.: 3.50, não 3,50)</t>
+          <t xml:space="preserve">  • data_validade — formato AAAA-MM-DD (ex.: 2027-01-15); deixe em branco se o item não vence</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
+          <t xml:space="preserve">  • valor_unitario — número com ponto decimal (ex.: 3.50, não 3,50)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
           <t xml:space="preserve">  • numero_nota_fiscal — texto</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="9" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">  • fabricante — texto (ex.: 3M, Descarpack); vira o cadastro do ITEM, não do lote</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="6" t="inlineStr"/>
-    </row>
     <row r="31">
-      <c r="A31" s="6" t="inlineStr">
-        <is>
-          <t>As linhas 2 a 5 (fundo amarelo) são EXEMPLOS de preenchimento — apague-as antes de importar</t>
-        </is>
-      </c>
+      <c r="A31" s="6" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>de verdade, ou deixe (o script pula automaticamente porque esses códigos já existem no</t>
+          <t>As linhas 2 a 5 (fundo amarelo) são EXEMPLOS de preenchimento — apague-as antes de importar</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
+          <t>de verdade, ou deixe (o script pula automaticamente porque esses códigos já existem no</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
           <t>catálogo de exemplo do ambiente de teste).</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="6" t="inlineStr"/>
-    </row>
     <row r="35">
-      <c r="A35" s="7" t="inlineStr">
+      <c r="A35" s="6" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="7" t="inlineStr">
         <is>
           <t>COMO RODAR (a partir da pasta backend/, com o ambiente já configurado):</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="6" t="inlineStr"/>
-    </row>
     <row r="37">
-      <c r="A37" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  python scripts/importar_itens_planilha.py caminho/modelo_importacao_itens.xlsx \</t>
-        </is>
-      </c>
+      <c r="A37" s="6" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
+          <t xml:space="preserve">  python scripts/importar_itens_planilha.py caminho/modelo_importacao_itens.xlsx \</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="inlineStr">
+        <is>
           <t xml:space="preserve">      --api-url http://localhost:8000 --login coordenador --senha "sua-senha"</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="6" t="inlineStr"/>
-    </row>
     <row r="40">
-      <c r="A40" s="6" t="inlineStr">
-        <is>
-          <t>Ver docs/05_INSTALACAO_SERVIDOR_LOCAL.md para o passo completo dentro do processo de</t>
-        </is>
-      </c>
+      <c r="A40" s="6" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
+        <is>
+          <t>Ver docs/05_INSTALACAO_SERVIDOR_LOCAL.md para o passo completo dentro do processo de</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="6" t="inlineStr">
         <is>
           <t>instalação.</t>
         </is>

</xml_diff>

<commit_message>
Adiciona categoria 'Enxoval' ao cadastro de item
5a categoria fixa (roupa de cama/hospitalar) -- diferente das outras
adicoes de enum desta sessao, a constraint categoria_item_enum foi
criada de verdade na migracao 0004 (nao e o bug do Enum inline), entao
0008 precisa dropar e recriar a constraint em vez de so criar.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/modelo_importacao_itens.xlsx
+++ b/docs/modelo_importacao_itens.xlsx
@@ -1033,7 +1033,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A42"/>
+  <dimension ref="A1:A43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -1147,155 +1147,162 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="inlineStr"/>
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Enxoval  →  roupa de cama/hospitalar (lençol, fronha, avental de tecido, etc.)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="inlineStr">
-        <is>
-          <t>COLUNAS OPCIONAIS (fundo verde no cabeçalho — preencha só se já tiver estoque desse item</t>
-        </is>
-      </c>
+      <c r="A19" s="6" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
+          <t>COLUNAS OPCIONAIS (fundo verde no cabeçalho — preencha só se já tiver estoque desse item</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
           <t>pra registrar junto com o cadastro; deixando em branco, o item nasce com saldo 0 e dá pra</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="7" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
         <is>
           <t>"dar entrada" depois pela tela Entrada por Compra. estoque_minimo e fabricante são</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="9" t="inlineStr">
-        <is>
-          <t>as exceções: não têm relação com estoque, são só dados a mais do cadastro do item,</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="9" t="inlineStr">
         <is>
-          <t>sempre opcionais):</t>
+          <t>as exceções: não têm relação com estoque, são só dados a mais do cadastro do item,</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="9" t="inlineStr">
         <is>
+          <t>sempre opcionais):</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="9" t="inlineStr">
+        <is>
           <t xml:space="preserve">  • estoque_minimo — número inteiro; 0 se deixar em branco ou preencher algo que não é número</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • quantidade — número inteiro; SE preenchida, cria automaticamente uma entrada de estoque</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • numero_lote — texto, opcional mesmo com quantidade preenchida</t>
+          <t xml:space="preserve">  • quantidade — número inteiro; SE preenchida, cria automaticamente uma entrada de estoque</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • data_validade — formato AAAA-MM-DD (ex.: 2027-01-15); deixe em branco se o item não vence</t>
+          <t xml:space="preserve">  • numero_lote — texto, opcional mesmo com quantidade preenchida</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • valor_unitario — número com ponto decimal (ex.: 3.50, não 3,50)</t>
+          <t xml:space="preserve">  • data_validade — formato AAAA-MM-DD (ex.: 2027-01-15); deixe em branco se o item não vence</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
+          <t xml:space="preserve">  • valor_unitario — número com ponto decimal (ex.: 3.50, não 3,50)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
           <t xml:space="preserve">  • numero_nota_fiscal — texto</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="9" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">  • fabricante — texto (ex.: 3M, Descarpack); vira o cadastro do ITEM, não do lote</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="6" t="inlineStr"/>
-    </row>
     <row r="32">
-      <c r="A32" s="6" t="inlineStr">
-        <is>
-          <t>As linhas 2 a 5 (fundo amarelo) são EXEMPLOS de preenchimento — apague-as antes de importar</t>
-        </is>
-      </c>
+      <c r="A32" s="6" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>de verdade, ou deixe (o script pula automaticamente porque esses códigos já existem no</t>
+          <t>As linhas 2 a 5 (fundo amarelo) são EXEMPLOS de preenchimento — apague-as antes de importar</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
+          <t>de verdade, ou deixe (o script pula automaticamente porque esses códigos já existem no</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="inlineStr">
+        <is>
           <t>catálogo de exemplo do ambiente de teste).</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="6" t="inlineStr"/>
-    </row>
     <row r="36">
-      <c r="A36" s="7" t="inlineStr">
+      <c r="A36" s="6" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="7" t="inlineStr">
         <is>
           <t>COMO RODAR (a partir da pasta backend/, com o ambiente já configurado):</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="6" t="inlineStr"/>
-    </row>
     <row r="38">
-      <c r="A38" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  python scripts/importar_itens_planilha.py caminho/modelo_importacao_itens.xlsx \</t>
-        </is>
-      </c>
+      <c r="A38" s="6" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
+          <t xml:space="preserve">  python scripts/importar_itens_planilha.py caminho/modelo_importacao_itens.xlsx \</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="inlineStr">
+        <is>
           <t xml:space="preserve">      --api-url http://localhost:8000 --login coordenador --senha "sua-senha"</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="6" t="inlineStr"/>
-    </row>
     <row r="41">
-      <c r="A41" s="6" t="inlineStr">
-        <is>
-          <t>Ver docs/05_INSTALACAO_SERVIDOR_LOCAL.md para o passo completo dentro do processo de</t>
-        </is>
-      </c>
+      <c r="A41" s="6" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
+        <is>
+          <t>Ver docs/05_INSTALACAO_SERVIDOR_LOCAL.md para o passo completo dentro do processo de</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="6" t="inlineStr">
         <is>
           <t>instalação.</t>
         </is>

</xml_diff>